<commit_message>
add cs or vs in id b95b789f91bd18cb281137e7d3a21f1d1ab0ab95
</commit_message>
<xml_diff>
--- a/ig/nr-add-marital-status-binding/StructureDefinition-fr-core-patient-ins.xlsx
+++ b/ig/nr-add-marital-status-binding/StructureDefinition-fr-core-patient-ins.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-01-25T10:58:01+00:00</t>
+    <t>2024-01-29T09:41:10+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -2219,7 +2219,7 @@
     <t>Most, if not all systems capture it.</t>
   </si>
   <si>
-    <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-marital-status</t>
+    <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-marital-status</t>
   </si>
   <si>
     <t>player[classCode=PSN]/maritalStatusCode</t>

</xml_diff>